<commit_message>
Fix internal hyperlinks: use Hyperlink(location=) not target='#...'
Also name the tabs in the intro text so the sheets read correctly even where the
viewer disables link navigation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_wide_long.xlsx
+++ b/textbook_examples/mod01_wide_long.xlsx
@@ -493,7 +493,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The next two tabs hold exactly the same numbers — three rural municipalities, three crops, one year — laid out two different ways.  Open them side by side and compare.</t>
+          <t>The next two tabs — Wide and Long — hold exactly the same numbers: three rural municipalities, three crops, one year, laid out two different ways.  Use the tabs along the bottom of the window to switch between them.</t>
         </is>
       </c>
     </row>
@@ -550,8 +550,8 @@
     <mergeCell ref="A8:E8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId2"/>
+    <hyperlink ref="A4" location="'Wide'!A1"/>
+    <hyperlink ref="A6" location="'Long'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>